<commit_message>
Mean to Median Correction
</commit_message>
<xml_diff>
--- a/Dataset_limpio.xlsx
+++ b/Dataset_limpio.xlsx
@@ -573,7 +573,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1113,7 +1113,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1637,7 +1637,7 @@
         <v>22</v>
       </c>
       <c r="AA11" t="n">
-        <v>13207</v>
+        <v>10295</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
@@ -2085,7 +2085,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2193,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5109,7 +5109,7 @@
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -5217,7 +5217,7 @@
         <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -5309,7 +5309,7 @@
         <v>43</v>
       </c>
       <c r="AA45" t="n">
-        <v>13207</v>
+        <v>10295</v>
       </c>
       <c r="AB45" t="inlineStr">
         <is>
@@ -5325,7 +5325,7 @@
         <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -5417,7 +5417,7 @@
         <v>43</v>
       </c>
       <c r="AA46" t="n">
-        <v>13207</v>
+        <v>10295</v>
       </c>
       <c r="AB46" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
         <v>2</v>
       </c>
       <c r="C47" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -5649,7 +5649,7 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -5757,7 +5757,7 @@
         <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -7469,7 +7469,7 @@
         <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -8009,7 +8009,7 @@
         <v>-1</v>
       </c>
       <c r="C71" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -8225,7 +8225,7 @@
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -8333,7 +8333,7 @@
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
         <v>1</v>
       </c>
       <c r="C75" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -9197,7 +9197,7 @@
         <v>3</v>
       </c>
       <c r="C82" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -9305,7 +9305,7 @@
         <v>3</v>
       </c>
       <c r="C83" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -9413,7 +9413,7 @@
         <v>3</v>
       </c>
       <c r="C84" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -12113,7 +12113,7 @@
         <v>0</v>
       </c>
       <c r="C109" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -12221,7 +12221,7 @@
         <v>0</v>
       </c>
       <c r="C110" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -12545,7 +12545,7 @@
         <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -12653,7 +12653,7 @@
         <v>0</v>
       </c>
       <c r="C114" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -13733,7 +13733,7 @@
         <v>3</v>
       </c>
       <c r="C124" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -13949,7 +13949,7 @@
         <v>3</v>
       </c>
       <c r="C126" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -14057,7 +14057,7 @@
         <v>3</v>
       </c>
       <c r="C127" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -14165,7 +14165,7 @@
         <v>3</v>
       </c>
       <c r="C128" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -14273,7 +14273,7 @@
         <v>1</v>
       </c>
       <c r="C129" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -14365,7 +14365,7 @@
         <v>28</v>
       </c>
       <c r="AA129" t="n">
-        <v>13207</v>
+        <v>10295</v>
       </c>
       <c r="AB129" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         <v>0</v>
       </c>
       <c r="C130" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -14461,7 +14461,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="W130" t="n">
-        <v>13207</v>
+        <v>95</v>
       </c>
       <c r="X130" t="inlineStr"/>
       <c r="Y130" t="n">
@@ -14487,7 +14487,7 @@
         <v>2</v>
       </c>
       <c r="C131" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -14567,7 +14567,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="W131" t="n">
-        <v>13207</v>
+        <v>95</v>
       </c>
       <c r="X131" t="inlineStr"/>
       <c r="Y131" t="n">
@@ -19885,7 +19885,7 @@
         <v>-1</v>
       </c>
       <c r="C181" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
@@ -20749,7 +20749,7 @@
         <v>3</v>
       </c>
       <c r="C189" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
@@ -20965,7 +20965,7 @@
         <v>0</v>
       </c>
       <c r="C191" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
@@ -21073,7 +21073,7 @@
         <v>0</v>
       </c>
       <c r="C192" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
@@ -21181,7 +21181,7 @@
         <v>0</v>
       </c>
       <c r="C193" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>

</xml_diff>